<commit_message>
fix: pin trade offers while trading #489
- Block inventory changes and NPC dialogs while trading
- Reject offer changes after either side locks
- Verify offered items are still in place before exchange
- Add trade blocked and already locked messages to const string table
- Regenerate model code
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -1,32 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="8" activeTab="8" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="string.game.asset" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="string.game.bulletin" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="string.game.character" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="string.game.clan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="string.game.communication" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="string.game.door" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="string.game.equipment" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="string.game.etc" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="string.game.exception" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="string.game.group" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="string.game.item" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="string.game.map" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="string.game.mix" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="string.game.money" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="string.game.ride" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="string.game.spell" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="string.game.storage" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="string.game.trade" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="string.game.ui" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="string.gateway" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="string.login" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.asset" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.bulletin" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.character" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.clan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.communication" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.door" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.equipment" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.etc" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.exception" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.group" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.item" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.map" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.mix" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.money" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.ride" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.spell" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.storage" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.trade" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.game.ui" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.gateway" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="string.login" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -2770,7 +2770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3084,6 +3084,50 @@
       <c r="D14" s="1" t="inlineStr">
         <is>
           <t>{}님과 너무 멀리 떨어져 있습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>MESSAGE_TRADE_BLOCKED_WHILE_TRADING</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>교환 중에는 할 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MESSAGE_TRADE_ALREADY_LOCKED</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>확인을 누른 뒤에는 변경할 수 없습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: escrow items and money during marketplace listing
- Add ABORTED listing state, abort-list API and atomic archive move
- Store escrowed items in the item table with listing id and locked money
- Lock, deduct and unlock escrow in game items and money capacity checks
- Keep pending listings locked and settle them on a restore timer and login
- Refuse locked items in drop, throw, give, use and info handlers
- Validate the item model id when confirming a listing
- Add DB migrations, protocol schemas and generated code
- Add pending and locked item messages to const.string table
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -5303,7 +5303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D66"/>
+  <dimension ref="A1:D68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6761,6 +6761,50 @@
       <c r="D66" s="1" t="inlineStr">
         <is>
           <t>조합할 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_ITEM_LOCKED</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>거래소 등록 처리 중인 아이템입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_LISTING_PENDING</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>거래소 등록 결과를 확인하고 있습니다. 확인이 끝나면 자동으로 반영됩니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: resolve grok review findings FB-159 to FB-162
- Marketplace: purchase pending entry, abort-purchase tombstone and restore grace
- Marketplace: request deadline enforced before list/purchase commit
- Marketplace: drop purchase cascade FK, remove get-purchases
- Add MARKETPLACE_REQUEST_EXPIRED and purchase pending message tables
- Regenerate model and flatbuffer protocol
- Rezen: keep spawn table generation, rebuild after table reload
- Life: add attacker-less damage for scripts (spell 3049, 3059)
- Add HTTP hold test hook and marketplace recovery integration tests
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -5303,7 +5303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6805,6 +6805,28 @@
       <c r="D68" t="inlineStr">
         <is>
           <t>거래소 등록 결과를 확인하고 있습니다. 확인이 끝나면 자동으로 반영됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_PURCHASE_PENDING</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>거래소 구매 결과를 확인하고 있습니다. 확인이 끝나면 자동으로 반영됩니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add 6.51 reputation evaluation
- Handle C2S 0x46 reputation evaluation for 6.51 clients on the same game server
- Grant evaluation tickets every 12h of playtime up to 2 via evaluation_timer
- Block re-evaluating the same character within 24h
- Persist reputation, evaluation and evaluation_state (playtime and recent targets) in the user table
- Add EvaluatedTarget and Character evaluation fields to the internal protocol and regenerate code
- Add reputation constants and messages to const tables and regenerate model
- Add /인품설정 and /평가권설정 commands with Lua reputation/evaluation builtins
- Regenerate bot integration protocol registry
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -3883,7 +3883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4043,6 +4043,182 @@
       <c r="D7" s="1" t="inlineStr">
         <is>
           <t>경험치를 {} 잃었습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MESSAGE_REPUTATION_NO_EVALUATION</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>인품 평가권이 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MESSAGE_REPUTATION_ALREADY_EVALUATED</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>같은 사람은 하루에 한 번만 평가할 수 있습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MESSAGE_REPUTATION_SELF</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>자기 자신은 평가할 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MESSAGE_REPUTATION_RAISED</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>{}님의 인품을 올렸습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MESSAGE_REPUTATION_LOWERED</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>{}님의 인품을 내렸습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>MESSAGE_REPUTATION_RAISED_BY_OTHER</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>누군가 당신의 인품을 올렸습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>MESSAGE_REPUTATION_LOWERED_BY_OTHER</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>누군가 당신의 인품을 내렸습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>MESSAGE_REPUTATION_EVALUATION_GAINED</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>인품 평가권을 얻었습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: limit password brute force attempts #592
- Lock accounts for 10 minutes after 5 wrong passwords or birthdays
- Add ACCOUNT_LOCKED error code and message
- Rate limit login and change password handlers
- Close connections after repeated failures on one session
- Ignore password requests before session data exists
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -3533,7 +3533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3869,6 +3869,28 @@
       <c r="D15" s="1" t="inlineStr">
         <is>
           <t>이미 존재하는 이름입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MESSAGE_ACCOUNT_LOCKED</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>비밀번호를 여러 번 틀렸습니다. 잠시 후 다시 시도해 주세요.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: cap clans at 100 members
- Add clan MAX_MEMBER, CLAN_FULL_MEMBER and its message to the tables
- Reject a join when the clan is full and show the message in game
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -4277,7 +4277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4833,6 +4833,28 @@
       <c r="D25" t="inlineStr">
         <is>
           <t>문파에 가입하지 않았습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_FULL_MEMBER</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>문파 인원이 가득 찼습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: add messages and codes #769 #770 #773 #774
- const.string: clan self kick/role, invalid role, kick master, role names, marketplace rejection reasons
- enum.error: STORAGE_BOX_NOT_FOUND, STORAGE_BOX_ALREADY_RECEIVED, STORAGE_BOX_EXPIRED, CLAN_CANNOT_KICK_MASTER
- model: regenerate model.h and Model.cs
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -4277,7 +4277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4855,6 +4855,182 @@
       <c r="D26" t="inlineStr">
         <is>
           <t>문파 인원이 가득 찼습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_CANNOT_KICK_SELF</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>자기 자신은 축출할 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_CANNOT_CHANGE_ROLE_SELF</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>자기 자신의 직책은 변경할 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_INVALID_ROLE</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>잘못된 직책입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_ROLE_MATE</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>문원</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_ROLE_OFFICER</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>간부</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_ROLE_DEPUTY</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>부문주</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_ROLE_MASTER</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>문주</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_CANNOT_KICK_MASTER</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>문주는 축출할 수 없습니다.</t>
         </is>
       </c>
     </row>
@@ -5545,7 +5721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7069,6 +7245,160 @@
       <c r="D69" t="inlineStr">
         <is>
           <t>거래소 구매 결과를 확인하고 있습니다. 확인이 끝나면 자동으로 반영됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_LISTING_EXPIRED</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>등록 기간이 끝난 물품입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_LISTING_ALREADY_SOLD</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>이미 판매된 물품입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_LISTING_ALREADY_CANCELLED</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>이미 등록이 취소된 물품입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_INSUFFICIENT_STOCK</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>남은 수량이 부족합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_LISTING_LIMIT_EXCEEDED</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>더 이상 물품을 등록할 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_ITEM_NOT_TRADEABLE</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>거래소에 등록할 수 없는 아이템입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>MESSAGE_MARKETPLACE_NOT_LISTING_OWNER</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>본인이 등록한 물품이 아닙니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: add clan and match messages #789 #803
- const.string: MESSAGE_CLAN_NAME_INVALID, MESSAGE_CLAN_TITLE_INVALID, MESSAGE_MATCH_ALREADY_CLOSED
- model: regenerate model.h and Model.cs
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -4277,7 +4277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5031,6 +5031,50 @@
       <c r="D34" t="inlineStr">
         <is>
           <t>문주는 축출할 수 없습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_NAME_INVALID</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>사용할 수 없는 문파 이름입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_TITLE_INVALID</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>사용할 수 없는 문파 칭호입니다.</t>
         </is>
       </c>
     </row>
@@ -5721,7 +5765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D76"/>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7399,6 +7443,28 @@
       <c r="D76" t="inlineStr">
         <is>
           <t>본인이 등록한 물품이 아닙니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>MESSAGE_MATCH_ALREADY_CLOSED</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>이미 끝난 매치입니다. 원래 있던 곳으로 돌아갑니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: translate clan diplomacy errors #825
- const.string: add MESSAGE_CLAN_TARGET_ALREADY_ALLIED and regenerate the C++ and C# models
- clan actions: refuse an ally request when the target already has an ally
- clan events: map the diplomacy error codes to their messages
- clan_npc: stop the ally menu early when the target clan is allied
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -4277,7 +4277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5075,6 +5075,28 @@
       <c r="D36" t="inlineStr">
         <is>
           <t>사용할 수 없는 문파 칭호입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_TARGET_ALREADY_ALLIED</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>상대 문파는 이미 동맹을 맺은 문파가 있습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: hide HTTP errors from chat senders #970
- http: throw fb::http_error for HTTP request failures
- game: whisper and clan, group and friend chat log HTTP failures and show a Korean unconfirmed message
- data: add MESSAGE_CHAT_UNCONFIRMED and regenerate models
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -5111,7 +5111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5227,6 +5227,28 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>[친구] {}님이 접속하셨습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MESSAGE_CHAT_UNCONFIRMED</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>메시지 전달 여부를 확인하지 못했습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: hide HTTP errors on bulletin and group #970
- game: bulletin, mail and group actions log HTTP failures and show a Korean unconfirmed message instead of the internal error text
- data: add MESSAGE_REQUEST_UNCONFIRMED and regenerate models
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -5809,7 +5809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D77"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7509,6 +7509,28 @@
       <c r="D77" t="inlineStr">
         <is>
           <t>이미 끝난 매치입니다. 원래 있던 곳으로 돌아갑니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>MESSAGE_REQUEST_UNCONFIRMED</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>요청 결과를 확인하지 못했습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update table data #1002 #1005 #1006
- tables: add the BIRTHDAY_LOCKED error with its login message, remove the LOCK_WALK_SPEED option, add the clan invite-self message and reword the already-joined clan message; regenerate the C++ and C# models
</commit_message>
<xml_diff>
--- a/resources/table/const.string.xlsx
+++ b/resources/table/const.string.xlsx
@@ -3555,7 +3555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3913,6 +3913,28 @@
       <c r="D16" t="inlineStr">
         <is>
           <t>비밀번호를 여러 번 틀렸습니다. 잠시 후 다시 시도해 주세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MESSAGE_ACCOUNT_BIRTHDAY_LOCKED</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>생년월일을 여러 번 틀려 비밀번호 변경이 잠겼습니다. 24시간 뒤 다시 시도해 주세요.</t>
         </is>
       </c>
     </row>
@@ -4277,7 +4299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5097,6 +5119,28 @@
       <c r="D37" t="inlineStr">
         <is>
           <t>상대 문파는 이미 동맹을 맺은 문파가 있습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>MESSAGE_CLAN_CANNOT_INVITE_SELF</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>server</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>자기 자신은 등용할 수 없습니다.</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6078,7 @@
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>클랜 이미 있음</t>
+          <t>이미 문파에 가입되어 있습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>